<commit_message>
save: PRD review snapshot (in progress, file open in Excel)
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-PRD-v1.0-2026-06-30.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-PRD-v1.0-2026-06-30.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/palakjain/Vibe_Coding/finwise/docs/FCC-core-55-70/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE75F72-C541-474F-8AFC-D98C56AD24F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5AA3619-2A68-3A41-BD9F-A57F77998EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8340" yWindow="0" windowWidth="25260" windowHeight="19880" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6370" uniqueCount="2508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6371" uniqueCount="2509">
   <si>
     <t>Section</t>
   </si>
@@ -8165,6 +8165,9 @@
   </si>
   <si>
     <t>Is user providing TTM ROI on particular asset? If yes, why it say not editable?</t>
+  </si>
+  <si>
+    <t>Which kind T-bills will be? And what is HYSA?</t>
   </si>
 </sst>
 </file>
@@ -8361,6 +8364,12 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -8370,12 +8379,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9027,151 +9030,151 @@
       <c r="B14" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="D14" s="19"/>
-      <c r="E14" s="20"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="22"/>
     </row>
     <row r="15" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="19"/>
-      <c r="E15" s="20"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="22"/>
     </row>
     <row r="16" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="D16" s="19"/>
-      <c r="E16" s="20"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="22"/>
     </row>
     <row r="17" spans="2:5" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="D17" s="19"/>
-      <c r="E17" s="20"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="22"/>
     </row>
     <row r="18" spans="2:5" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="D18" s="19"/>
-      <c r="E18" s="20"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="22"/>
     </row>
     <row r="19" spans="2:5" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="D19" s="19"/>
-      <c r="E19" s="20"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="22"/>
     </row>
     <row r="20" spans="2:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="D20" s="19"/>
-      <c r="E20" s="20"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="22"/>
     </row>
     <row r="21" spans="2:5" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="D21" s="19"/>
-      <c r="E21" s="20"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="22"/>
     </row>
     <row r="22" spans="2:5" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="D22" s="19"/>
-      <c r="E22" s="20"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="22"/>
     </row>
     <row r="23" spans="2:5" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="D23" s="19"/>
-      <c r="E23" s="20"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="22"/>
     </row>
     <row r="24" spans="2:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="D24" s="19"/>
-      <c r="E24" s="20"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="22"/>
     </row>
     <row r="25" spans="2:5" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="D25" s="19"/>
-      <c r="E25" s="20"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="22"/>
     </row>
     <row r="26" spans="2:5" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="D26" s="19"/>
-      <c r="E26" s="20"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="22"/>
     </row>
     <row r="27" spans="2:5" ht="67.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="D27" s="19"/>
-      <c r="E27" s="20"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="22"/>
     </row>
     <row r="28" spans="2:5" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="20"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -9253,7 +9256,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>99</v>
       </c>
@@ -9290,7 +9293,7 @@
       <c r="L2" s="7"/>
       <c r="M2" s="7"/>
     </row>
-    <row r="3" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>110</v>
       </c>
@@ -9327,7 +9330,7 @@
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
     </row>
-    <row r="4" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>121</v>
       </c>
@@ -9364,7 +9367,7 @@
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
     </row>
-    <row r="5" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>132</v>
       </c>
@@ -9401,7 +9404,7 @@
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
     </row>
-    <row r="6" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>143</v>
       </c>
@@ -9438,7 +9441,7 @@
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
     </row>
-    <row r="7" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>154</v>
       </c>
@@ -9475,7 +9478,7 @@
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
     </row>
-    <row r="8" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>165</v>
       </c>
@@ -9512,7 +9515,7 @@
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
     </row>
-    <row r="9" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>176</v>
       </c>
@@ -9549,7 +9552,7 @@
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
     </row>
-    <row r="10" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>186</v>
       </c>
@@ -9586,7 +9589,7 @@
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
     </row>
-    <row r="11" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>197</v>
       </c>
@@ -9623,7 +9626,7 @@
       <c r="L11" s="7"/>
       <c r="M11" s="7"/>
     </row>
-    <row r="12" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>208</v>
       </c>
@@ -12091,7 +12094,7 @@
     <col min="9" max="9" width="22" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="30" customWidth="1"/>
-    <col min="12" max="12" width="16.33203125" style="24" customWidth="1"/>
+    <col min="12" max="12" width="16.33203125" style="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
@@ -12128,7 +12131,7 @@
       <c r="K1" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="L1" s="23" t="s">
+      <c r="L1" s="18" t="s">
         <v>2506</v>
       </c>
     </row>
@@ -12166,7 +12169,7 @@
       <c r="K2" s="12" t="s">
         <v>426</v>
       </c>
-      <c r="L2" s="24" t="s">
+      <c r="L2" s="19" t="s">
         <v>2507</v>
       </c>
     </row>
@@ -12553,6 +12556,9 @@
       </c>
       <c r="K13" s="12" t="s">
         <v>481</v>
+      </c>
+      <c r="L13" s="19" t="s">
+        <v>2508</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="108" customHeight="1" x14ac:dyDescent="0.2">
@@ -29712,14 +29718,14 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="23" t="s">
         <v>2397</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
     </row>
     <row r="3" spans="1:6" ht="121.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
@@ -29964,7 +29970,7 @@
         <v>2451</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>2452</v>
       </c>

</xml_diff>